<commit_message>
feat: Add web interface, export functionality, and update configurations
- Add web interface for managing prospects and viewing stats
- Add export functionality for prospect data
- Update email sequences and prospect data
- Remove outdated documentation files
- Update dependencies and CLI improvements
</commit_message>
<xml_diff>
--- a/data/prospects.xlsx
+++ b/data/prospects.xlsx
@@ -8,22 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gowustl-my.sharepoint.com/personal/lalakiya_wustl_edu/Documents/Neha/Cold-Email/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="11_2B59185F95A909F64819C7D0471510344D07F170" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABE5D100-990C-1A4C-8BC0-D6198D7D2C95}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_23786C507DE706BE4301A3C5BCCA6D90B7833691" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{079682E4-FA23-AF47-A496-8218AA34B48C}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="19880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="19880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Prospects" sheetId="1" r:id="rId1"/>
+    <sheet name="NO RESPONSE" sheetId="2" r:id="rId2"/>
+    <sheet name="RESPONSE" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Prospects!$A$1:$G$4</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="16">
   <si>
     <t>prospect_id</t>
   </si>
@@ -46,77 +45,41 @@
     <t>sequence_id</t>
   </si>
   <si>
-    <t>PROS-001</t>
-  </si>
-  <si>
-    <t>PROS-002</t>
-  </si>
-  <si>
-    <t>PROS-003</t>
-  </si>
-  <si>
-    <t>aggressive</t>
-  </si>
-  <si>
-    <t>RES-001</t>
-  </si>
-  <si>
-    <t>com1</t>
-  </si>
-  <si>
-    <t>RES-002</t>
-  </si>
-  <si>
-    <t>RES-003</t>
-  </si>
-  <si>
-    <t>role1</t>
-  </si>
-  <si>
-    <t>role2</t>
-  </si>
-  <si>
-    <t>role3</t>
-  </si>
-  <si>
-    <t>com2</t>
-  </si>
-  <si>
-    <t>com3</t>
-  </si>
-  <si>
-    <t>name1</t>
-  </si>
-  <si>
-    <t>name2</t>
-  </si>
-  <si>
-    <t>name3</t>
-  </si>
-  <si>
-    <t>shivamlalakiya151299@gmail.com</t>
-  </si>
-  <si>
-    <t>shivamlalakiya1@gmail.com</t>
-  </si>
-  <si>
-    <t>sutariyaneha30@gmail.com</t>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Company</t>
+  </si>
+  <si>
+    <t>Resume ID</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>total emails</t>
+  </si>
+  <si>
+    <t>first email sent</t>
+  </si>
+  <si>
+    <t>last email sent</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -130,12 +93,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -150,9 +119,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -168,10 +140,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -459,7 +427,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -494,77 +462,118 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="38" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="9" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="9" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="21" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="I1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="2" customWidth="1"/>
+    <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix dry-run mode and resume path handling
- Fix dry-run mode to not update database state (status, followup_step, etc.)
- Prevent event log creation in dry-run mode
- Fix resume path handling in web app (correct unpacking of find_resume_file)
- Add fallback to find resume by resume_id if resume_path is missing
- Fix sequence structure mismatch in web app (pass full structure to orchestrator)
- Fix MessageEvent.created_at references to use occurred_at instead
- Ensure all 3 emails (initial + 2 followups) are sent before marking as COMPLETED
</commit_message>
<xml_diff>
--- a/data/prospects.xlsx
+++ b/data/prospects.xlsx
@@ -1,108 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gowustl-my.sharepoint.com/personal/lalakiya_wustl_edu/Documents/Neha/Cold-Email/data/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_23786C507DE706BE4301A3C5BCCA6D90B7833691" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{079682E4-FA23-AF47-A496-8218AA34B48C}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="19880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="19880" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prospects" sheetId="1" r:id="rId1"/>
-    <sheet name="NO RESPONSE" sheetId="2" r:id="rId2"/>
-    <sheet name="RESPONSE" sheetId="3" r:id="rId3"/>
+    <sheet name="Prospects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="NO RESPONSE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="RESPONSE" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="16">
-  <si>
-    <t>prospect_id</t>
-  </si>
-  <si>
-    <t>full_name</t>
-  </si>
-  <si>
-    <t>company</t>
-  </si>
-  <si>
-    <t>email</t>
-  </si>
-  <si>
-    <t>resume_id</t>
-  </si>
-  <si>
-    <t>role_title</t>
-  </si>
-  <si>
-    <t>sequence_id</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Company</t>
-  </si>
-  <si>
-    <t>Resume ID</t>
-  </si>
-  <si>
-    <t>Role</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>total emails</t>
-  </si>
-  <si>
-    <t>first email sent</t>
-  </si>
-  <si>
-    <t>last email sent</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.34998626667073579"/>
+        <fgColor theme="0" tint="-0.3499862666707358"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -120,25 +62,84 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -426,40 +427,58 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13" bestFit="1" customWidth="1"/>
+    <col width="12.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="11.1640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="11.5" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="28.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="11.5" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="17" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="13" bestFit="1" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>prospect_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>full_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>resume_id</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>role_title</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>sequence_id</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -468,53 +487,78 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="38" customWidth="1"/>
-    <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="9" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="9" customWidth="1"/>
-    <col min="8" max="8" width="11" customWidth="1"/>
-    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="21" customWidth="1"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="14" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>15</v>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resume ID</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>total emails</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>first email sent</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>last email sent</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -523,54 +567,133 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="2" customWidth="1"/>
-    <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17" bestFit="1" customWidth="1"/>
+    <col width="38" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="32" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="17" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="9" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="11" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="14" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="14" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="21" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="21" bestFit="1" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>15</v>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resume ID</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>total emails</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>first email sent</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>last email sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>133c6879-ad1a-4f7a-990c-d7f72fe67d8b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>shivamlalakiya151299@gmail.com</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Shivam Lalakiya</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>WashU</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>RES-001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Data Analyst</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>REPLIED</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-01-17 23:26:53</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-01-17 23:26:01</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>